<commit_message>
fix(leads-deploy): diagnosticar rechazos y evitar CRM falso
</commit_message>
<xml_diff>
--- a/backend/data/Programas_UTEL_Todos_los_Paises.xlsx
+++ b/backend/data/Programas_UTEL_Todos_los_Paises.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="México" sheetId="1" r:id="Rab219a6509d24c97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Argentina" sheetId="2" r:id="Red616b0de2a6495c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colombia" sheetId="3" r:id="R23087300d3524154"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perú" sheetId="4" r:id="Re75c73e4d40b4cf0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ecuador" sheetId="5" r:id="R962a1485113644e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="USA" sheetId="6" r:id="R401749cd67ff4d1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bolivia" sheetId="7" r:id="R801c1c783ed04e56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chile" sheetId="8" r:id="R0f130f586d9640fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rep. Dominicana" sheetId="9" r:id="R3c44cf035e344e91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guatemala" sheetId="10" r:id="R4492c4cd422d4573"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panamá" sheetId="11" r:id="R262bb3361dd3410f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="El Salvador" sheetId="12" r:id="Rc9291afbe741490a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Philippines" sheetId="13" r:id="R72dcbcf7842b4926"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indonesia" sheetId="14" r:id="Rbec1ca992f5a4a9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paraguay" sheetId="15" r:id="Rc67221567fe349bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="México" sheetId="1" r:id="Rded5deab0b20458c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Argentina" sheetId="2" r:id="Rdb3423d586694d99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colombia" sheetId="3" r:id="R5042ba6aca334954"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perú" sheetId="4" r:id="R2461a00554ac4e20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ecuador" sheetId="5" r:id="R673ef71e4f624036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="USA" sheetId="6" r:id="Rb34ffccb57294fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bolivia" sheetId="7" r:id="R2222c3979f17489e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chile" sheetId="8" r:id="Rb2b78b9a374840f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rep. Dominicana" sheetId="9" r:id="R403f9ceaec124ccf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guatemala" sheetId="10" r:id="Racecad5230ff40dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panamá" sheetId="11" r:id="R1e04af048ee24241"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="El Salvador" sheetId="12" r:id="R86ccfec85ffa495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Philippines" sheetId="13" r:id="R6531e83271104c49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indonesia" sheetId="14" r:id="R1d2443bfec874463"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paraguay" sheetId="15" r:id="R24ef9bf3851a408a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -113,54 +113,19 @@
     <x:border/>
     <x:border/>
     <x:border/>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2206,7 +2171,7 @@
         <x:v>Bachillerato en línea</x:v>
       </x:c>
       <x:c r="B124" s="110" t="str">
-        <x:v>Bachillerato General</x:v>
+        <x:v>Bachillerato en línea</x:v>
       </x:c>
       <x:c r="C124" s="111" t="str">
         <x:v>https://utel.edu.mx/bachillerato</x:v>
@@ -5328,7 +5293,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R066fe873a8724176"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43696a243d684a93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6027,7 +5992,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R524eb811fdb449e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc814b87bf5c24738"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6605,7 +6570,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27debda1366b4de1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d8f0b5a85c5428f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7293,7 +7258,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7a2c9014d5843d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b4165d3668e4c63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7475,7 +7440,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbac19b1ba344b24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R215632995c0a4e51"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7657,7 +7622,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61c93a4985644184"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49766e6aa7da4c9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8246,7 +8211,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8745b3676e741cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15177e0ebc9f4719"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9033,7 +8998,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d518fffe6f3494d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77f85df2d6114399"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11087,7 +11052,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79d7f108e32a4db2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdeb9ad0e7ff84d0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13051,7 +13016,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72844ed6d021498d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c97e15699074d9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14736,7 +14701,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b4dadf1656a4647"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ab645aad06d424f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15926,7 +15891,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8a82eb718ad4bac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R675b081a39b54082"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16520,7 +16485,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5aff260254347da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01c84190db644453"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17109,7 +17074,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R727f044b946149a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fda5aa72501436d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18339,7 +18304,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7a3ae0d5266492c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff00ee03e2524906"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>